<commit_message>
Clear example-row notes left on the operator's four SKUs
When the SKU column was overwritten with the operator's products, the
example rows' notes stayed behind, so ring R1794 read "earrings have no
size axis" and two Include = Y rows read "staged (Include = N)". Only
those four notes are cleared; dropdowns and header comments are intact
and `workbook validate` reports 4 rows, 0 errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Product Listing.xlsx
+++ b/Product Listing.xlsx
@@ -1219,11 +1219,7 @@
       </c>
       <c r="Z2" s="19" t="n"/>
       <c r="AA2" s="19" t="n"/>
-      <c r="AB2" s="19" t="inlineStr">
-        <is>
-          <t>Example row — delete or set Include=N once you add your own.</t>
-        </is>
-      </c>
+      <c r="AB2" s="19" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
@@ -1279,11 +1275,7 @@
       </c>
       <c r="Z3" s="19" t="n"/>
       <c r="AA3" s="19" t="n"/>
-      <c r="AB3" s="19" t="inlineStr">
-        <is>
-          <t>Example row — earrings have no size axis, so Variations = none.</t>
-        </is>
-      </c>
+      <c r="AB3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
@@ -1335,11 +1327,7 @@
       <c r="Y4" s="19" t="n"/>
       <c r="Z4" s="19" t="n"/>
       <c r="AA4" s="19" t="n"/>
-      <c r="AB4" s="19" t="inlineStr">
-        <is>
-          <t>Example row, staged (Include = N) so it is skipped.</t>
-        </is>
-      </c>
+      <c r="AB4" s="19" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
@@ -1391,11 +1379,7 @@
       <c r="Y5" s="19" t="n"/>
       <c r="Z5" s="19" t="n"/>
       <c r="AA5" s="19" t="n"/>
-      <c r="AB5" s="19" t="inlineStr">
-        <is>
-          <t>Example row, staged (Include = N) so it is skipped.</t>
-        </is>
-      </c>
+      <c r="AB5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n"/>

</xml_diff>